<commit_message>
Add plot data sheet
</commit_message>
<xml_diff>
--- a/passive_seismic/plot_data.xlsx
+++ b/passive_seismic/plot_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t xml:space="preserve">STATION</t>
   </si>
@@ -40,10 +40,13 @@
     <t xml:space="preserve">ELEVATION</t>
   </si>
   <si>
+    <t xml:space="preserve">f0 (Hz)</t>
+  </si>
+  <si>
     <t xml:space="preserve">A0</t>
   </si>
   <si>
-    <t xml:space="preserve">f0</t>
+    <t xml:space="preserve">Kg</t>
   </si>
   <si>
     <t xml:space="preserve">Vs30</t>
@@ -233,16 +236,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.000000000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -258,12 +263,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -313,19 +312,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -333,7 +332,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -460,7 +459,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:W61"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
@@ -500,10 +499,13 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>-7.74603882435985</v>
@@ -520,10 +522,26 @@
       <c r="F2" s="5" t="n">
         <v>191.163032529785</v>
       </c>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+      <c r="I2" s="0"/>
+      <c r="J2" s="0"/>
+      <c r="L2" s="0"/>
+      <c r="M2" s="0"/>
+      <c r="N2" s="0"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>-7.74663162231445</v>
@@ -540,10 +558,26 @@
       <c r="F3" s="5" t="n">
         <v>185.148940991211</v>
       </c>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0"/>
+      <c r="J3" s="0"/>
+      <c r="L3" s="0"/>
+      <c r="M3" s="0"/>
+      <c r="N3" s="0"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>-7.75365666666666</v>
@@ -560,10 +594,26 @@
       <c r="F4" s="5" t="n">
         <v>127.667381254395</v>
       </c>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0"/>
+      <c r="N4" s="0"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>-7.75709405564505</v>
@@ -580,10 +630,26 @@
       <c r="F5" s="5" t="n">
         <v>104.056293674316</v>
       </c>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+      <c r="I5" s="0"/>
+      <c r="J5" s="0"/>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0"/>
+      <c r="N5" s="0"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>-7.76309333333333</v>
@@ -600,10 +666,26 @@
       <c r="F6" s="5" t="n">
         <v>97.0373458862305</v>
       </c>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+      <c r="I6" s="0"/>
+      <c r="J6" s="0"/>
+      <c r="L6" s="0"/>
+      <c r="M6" s="0"/>
+      <c r="N6" s="0"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
+      <c r="W6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>-7.73740890654394</v>
@@ -620,10 +702,26 @@
       <c r="F7" s="5" t="n">
         <v>347.634552001953</v>
       </c>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0"/>
+      <c r="J7" s="0"/>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0"/>
+      <c r="N7" s="0"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>-7.738853</v>
@@ -640,10 +738,26 @@
       <c r="F8" s="5" t="n">
         <v>216.977668832031</v>
       </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+      <c r="I8" s="0"/>
+      <c r="J8" s="0"/>
+      <c r="L8" s="0"/>
+      <c r="M8" s="0"/>
+      <c r="N8" s="0"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="6"/>
+      <c r="W8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>-7.743</v>
@@ -660,10 +774,26 @@
       <c r="F9" s="5" t="n">
         <v>172.269851465332</v>
       </c>
+      <c r="G9" s="0"/>
+      <c r="H9" s="0"/>
+      <c r="I9" s="0"/>
+      <c r="J9" s="0"/>
+      <c r="L9" s="0"/>
+      <c r="M9" s="0"/>
+      <c r="N9" s="0"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="6"/>
+      <c r="V9" s="6"/>
+      <c r="W9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>-7.743479</v>
@@ -680,10 +810,26 @@
       <c r="F10" s="5" t="n">
         <v>112.366561804688</v>
       </c>
+      <c r="G10" s="0"/>
+      <c r="H10" s="0"/>
+      <c r="I10" s="0"/>
+      <c r="J10" s="0"/>
+      <c r="L10" s="0"/>
+      <c r="M10" s="0"/>
+      <c r="N10" s="0"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="6"/>
+      <c r="V10" s="6"/>
+      <c r="W10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>-7.74505401956837</v>
@@ -700,10 +846,26 @@
       <c r="F11" s="5" t="n">
         <v>111.736358530518</v>
       </c>
+      <c r="G11" s="0"/>
+      <c r="H11" s="0"/>
+      <c r="I11" s="0"/>
+      <c r="J11" s="0"/>
+      <c r="L11" s="0"/>
+      <c r="M11" s="0"/>
+      <c r="N11" s="0"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="6"/>
+      <c r="U11" s="6"/>
+      <c r="V11" s="6"/>
+      <c r="W11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>-7.74790333333333</v>
@@ -720,10 +882,26 @@
       <c r="F12" s="5" t="n">
         <v>99.3031997680664</v>
       </c>
+      <c r="G12" s="0"/>
+      <c r="H12" s="0"/>
+      <c r="I12" s="0"/>
+      <c r="J12" s="0"/>
+      <c r="L12" s="0"/>
+      <c r="M12" s="0"/>
+      <c r="N12" s="0"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="6"/>
+      <c r="U12" s="6"/>
+      <c r="V12" s="6"/>
+      <c r="W12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>-7.731415</v>
@@ -740,10 +918,26 @@
       <c r="F13" s="5" t="n">
         <v>282.519851674805</v>
       </c>
+      <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
+      <c r="I13" s="0"/>
+      <c r="J13" s="0"/>
+      <c r="L13" s="0"/>
+      <c r="M13" s="0"/>
+      <c r="N13" s="0"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
+      <c r="V13" s="6"/>
+      <c r="W13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>-7.73346</v>
@@ -760,10 +954,26 @@
       <c r="F14" s="5" t="n">
         <v>122.482795642578</v>
       </c>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0"/>
+      <c r="J14" s="0"/>
+      <c r="L14" s="0"/>
+      <c r="M14" s="0"/>
+      <c r="N14" s="0"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
+      <c r="V14" s="6"/>
+      <c r="W14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>-7.73511</v>
@@ -780,10 +990,26 @@
       <c r="F15" s="5" t="n">
         <v>112.215297560547</v>
       </c>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
+      <c r="L15" s="0"/>
+      <c r="M15" s="0"/>
+      <c r="N15" s="0"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6"/>
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
+      <c r="V15" s="6"/>
+      <c r="W15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>-7.73861166666666</v>
@@ -800,10 +1026,26 @@
       <c r="F16" s="5" t="n">
         <v>105.960304286133</v>
       </c>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
+      <c r="L16" s="0"/>
+      <c r="M16" s="0"/>
+      <c r="N16" s="0"/>
+      <c r="O16" s="6"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="6"/>
+      <c r="S16" s="6"/>
+      <c r="T16" s="6"/>
+      <c r="U16" s="6"/>
+      <c r="V16" s="6"/>
+      <c r="W16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>-7.74097385669832</v>
@@ -820,10 +1062,26 @@
       <c r="F17" s="5" t="n">
         <v>101.337562561035</v>
       </c>
+      <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
+      <c r="I17" s="0"/>
+      <c r="J17" s="0"/>
+      <c r="L17" s="0"/>
+      <c r="M17" s="0"/>
+      <c r="N17" s="0"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="6"/>
+      <c r="S17" s="6"/>
+      <c r="T17" s="6"/>
+      <c r="U17" s="6"/>
+      <c r="V17" s="6"/>
+      <c r="W17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>-7.72301666666666</v>
@@ -840,10 +1098,26 @@
       <c r="F18" s="5" t="n">
         <v>197.519668579102</v>
       </c>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
+      <c r="I18" s="0"/>
+      <c r="J18" s="0"/>
+      <c r="L18" s="0"/>
+      <c r="M18" s="0"/>
+      <c r="N18" s="0"/>
+      <c r="O18" s="6"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="6"/>
+      <c r="R18" s="6"/>
+      <c r="S18" s="6"/>
+      <c r="T18" s="6"/>
+      <c r="U18" s="6"/>
+      <c r="V18" s="6"/>
+      <c r="W18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>-7.725055</v>
@@ -860,10 +1134,26 @@
       <c r="F19" s="5" t="n">
         <v>142.18503559668</v>
       </c>
+      <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
+      <c r="I19" s="0"/>
+      <c r="J19" s="0"/>
+      <c r="L19" s="0"/>
+      <c r="M19" s="0"/>
+      <c r="N19" s="0"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="6"/>
+      <c r="S19" s="6"/>
+      <c r="T19" s="6"/>
+      <c r="U19" s="6"/>
+      <c r="V19" s="6"/>
+      <c r="W19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>-7.72724666666667</v>
@@ -880,10 +1170,26 @@
       <c r="F20" s="5" t="n">
         <v>116.86959079248</v>
       </c>
+      <c r="G20" s="0"/>
+      <c r="H20" s="0"/>
+      <c r="I20" s="0"/>
+      <c r="J20" s="0"/>
+      <c r="L20" s="0"/>
+      <c r="M20" s="0"/>
+      <c r="N20" s="0"/>
+      <c r="O20" s="6"/>
+      <c r="P20" s="6"/>
+      <c r="Q20" s="6"/>
+      <c r="R20" s="6"/>
+      <c r="S20" s="6"/>
+      <c r="T20" s="6"/>
+      <c r="U20" s="6"/>
+      <c r="V20" s="6"/>
+      <c r="W20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>-7.73107</v>
@@ -900,10 +1206,26 @@
       <c r="F21" s="5" t="n">
         <v>108.508556337646</v>
       </c>
+      <c r="G21" s="0"/>
+      <c r="H21" s="0"/>
+      <c r="I21" s="0"/>
+      <c r="J21" s="0"/>
+      <c r="L21" s="0"/>
+      <c r="M21" s="0"/>
+      <c r="N21" s="0"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="6"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="6"/>
+      <c r="U21" s="6"/>
+      <c r="V21" s="6"/>
+      <c r="W21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>-7.73054166666666</v>
@@ -920,10 +1242,26 @@
       <c r="F22" s="5" t="n">
         <v>95.2035522460938</v>
       </c>
+      <c r="G22" s="0"/>
+      <c r="H22" s="0"/>
+      <c r="I22" s="0"/>
+      <c r="J22" s="0"/>
+      <c r="L22" s="0"/>
+      <c r="M22" s="0"/>
+      <c r="N22" s="0"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="6"/>
+      <c r="S22" s="6"/>
+      <c r="T22" s="6"/>
+      <c r="U22" s="6"/>
+      <c r="V22" s="6"/>
+      <c r="W22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>-7.73295791631359</v>
@@ -940,10 +1278,26 @@
       <c r="F23" s="5" t="n">
         <v>113.839790344238</v>
       </c>
+      <c r="G23" s="0"/>
+      <c r="H23" s="0"/>
+      <c r="I23" s="0"/>
+      <c r="J23" s="0"/>
+      <c r="L23" s="0"/>
+      <c r="M23" s="0"/>
+      <c r="N23" s="0"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>-7.72960051265161</v>
@@ -960,10 +1314,26 @@
       <c r="F24" s="5" t="n">
         <v>136.683654851074</v>
       </c>
+      <c r="G24" s="0"/>
+      <c r="H24" s="0"/>
+      <c r="I24" s="0"/>
+      <c r="J24" s="0"/>
+      <c r="L24" s="0"/>
+      <c r="M24" s="0"/>
+      <c r="N24" s="0"/>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="6"/>
+      <c r="T24" s="6"/>
+      <c r="U24" s="6"/>
+      <c r="V24" s="6"/>
+      <c r="W24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>-7.74705</v>
@@ -980,10 +1350,26 @@
       <c r="F25" s="5" t="n">
         <v>106.308010254883</v>
       </c>
+      <c r="G25" s="0"/>
+      <c r="H25" s="0"/>
+      <c r="I25" s="0"/>
+      <c r="J25" s="0"/>
+      <c r="L25" s="0"/>
+      <c r="M25" s="0"/>
+      <c r="N25" s="0"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6"/>
+      <c r="R25" s="6"/>
+      <c r="S25" s="6"/>
+      <c r="T25" s="6"/>
+      <c r="U25" s="6"/>
+      <c r="V25" s="6"/>
+      <c r="W25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>-7.74886467967605</v>
@@ -1000,10 +1386,26 @@
       <c r="F26" s="5" t="n">
         <v>103.607296213867</v>
       </c>
+      <c r="G26" s="0"/>
+      <c r="H26" s="0"/>
+      <c r="I26" s="0"/>
+      <c r="J26" s="0"/>
+      <c r="L26" s="0"/>
+      <c r="M26" s="0"/>
+      <c r="N26" s="0"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="6"/>
+      <c r="S26" s="6"/>
+      <c r="T26" s="6"/>
+      <c r="U26" s="6"/>
+      <c r="V26" s="6"/>
+      <c r="W26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>-7.75520166666667</v>
@@ -1020,10 +1422,26 @@
       <c r="F27" s="5" t="n">
         <v>105.647788823486</v>
       </c>
+      <c r="G27" s="0"/>
+      <c r="H27" s="0"/>
+      <c r="I27" s="0"/>
+      <c r="J27" s="0"/>
+      <c r="L27" s="0"/>
+      <c r="M27" s="0"/>
+      <c r="N27" s="0"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6"/>
+      <c r="R27" s="6"/>
+      <c r="S27" s="6"/>
+      <c r="T27" s="6"/>
+      <c r="U27" s="6"/>
+      <c r="V27" s="6"/>
+      <c r="W27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>-7.751647823625</v>
@@ -1040,10 +1458,26 @@
       <c r="F28" s="5" t="n">
         <v>104.428081663086</v>
       </c>
+      <c r="G28" s="0"/>
+      <c r="H28" s="0"/>
+      <c r="I28" s="0"/>
+      <c r="J28" s="0"/>
+      <c r="L28" s="0"/>
+      <c r="M28" s="0"/>
+      <c r="N28" s="0"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+      <c r="R28" s="6"/>
+      <c r="S28" s="6"/>
+      <c r="T28" s="6"/>
+      <c r="U28" s="6"/>
+      <c r="V28" s="6"/>
+      <c r="W28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>-7.76167166666667</v>
@@ -1060,10 +1494,26 @@
       <c r="F29" s="5" t="n">
         <v>98.5598718918457</v>
       </c>
+      <c r="G29" s="0"/>
+      <c r="H29" s="0"/>
+      <c r="I29" s="0"/>
+      <c r="J29" s="0"/>
+      <c r="L29" s="0"/>
+      <c r="M29" s="0"/>
+      <c r="N29" s="0"/>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6"/>
+      <c r="R29" s="6"/>
+      <c r="S29" s="6"/>
+      <c r="T29" s="6"/>
+      <c r="U29" s="6"/>
+      <c r="V29" s="6"/>
+      <c r="W29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>-7.76939369418946</v>
@@ -1080,10 +1530,26 @@
       <c r="F30" s="5" t="n">
         <v>87.5125579833984</v>
       </c>
+      <c r="G30" s="0"/>
+      <c r="H30" s="0"/>
+      <c r="I30" s="0"/>
+      <c r="J30" s="0"/>
+      <c r="L30" s="0"/>
+      <c r="M30" s="0"/>
+      <c r="N30" s="0"/>
+      <c r="O30" s="6"/>
+      <c r="P30" s="6"/>
+      <c r="Q30" s="6"/>
+      <c r="R30" s="6"/>
+      <c r="S30" s="6"/>
+      <c r="T30" s="6"/>
+      <c r="U30" s="6"/>
+      <c r="V30" s="6"/>
+      <c r="W30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>-7.76240666666667</v>
@@ -1100,10 +1566,26 @@
       <c r="F31" s="5" t="n">
         <v>156.905288773438</v>
       </c>
+      <c r="G31" s="0"/>
+      <c r="H31" s="0"/>
+      <c r="I31" s="0"/>
+      <c r="J31" s="0"/>
+      <c r="L31" s="0"/>
+      <c r="M31" s="0"/>
+      <c r="N31" s="0"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+      <c r="T31" s="6"/>
+      <c r="U31" s="6"/>
+      <c r="V31" s="6"/>
+      <c r="W31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>-7.77120166666667</v>
@@ -1120,10 +1602,26 @@
       <c r="F32" s="5" t="n">
         <v>104.27709197998</v>
       </c>
+      <c r="G32" s="0"/>
+      <c r="H32" s="0"/>
+      <c r="I32" s="0"/>
+      <c r="J32" s="0"/>
+      <c r="L32" s="0"/>
+      <c r="M32" s="0"/>
+      <c r="N32" s="0"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6"/>
+      <c r="R32" s="6"/>
+      <c r="S32" s="6"/>
+      <c r="T32" s="6"/>
+      <c r="U32" s="6"/>
+      <c r="V32" s="6"/>
+      <c r="W32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>-7.77023</v>
@@ -1140,10 +1638,26 @@
       <c r="F33" s="5" t="n">
         <v>180.585647583008</v>
       </c>
+      <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
+      <c r="I33" s="0"/>
+      <c r="J33" s="0"/>
+      <c r="L33" s="0"/>
+      <c r="M33" s="0"/>
+      <c r="N33" s="0"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6"/>
+      <c r="R33" s="6"/>
+      <c r="S33" s="6"/>
+      <c r="T33" s="6"/>
+      <c r="U33" s="6"/>
+      <c r="V33" s="6"/>
+      <c r="W33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>-7.74059808306336</v>
@@ -1160,10 +1674,26 @@
       <c r="F34" s="5" t="n">
         <v>184.640991210938</v>
       </c>
+      <c r="G34" s="0"/>
+      <c r="H34" s="0"/>
+      <c r="I34" s="0"/>
+      <c r="J34" s="0"/>
+      <c r="L34" s="0"/>
+      <c r="M34" s="0"/>
+      <c r="N34" s="0"/>
+      <c r="O34" s="6"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6"/>
+      <c r="R34" s="6"/>
+      <c r="S34" s="6"/>
+      <c r="T34" s="6"/>
+      <c r="U34" s="6"/>
+      <c r="V34" s="6"/>
+      <c r="W34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>-7.729845</v>
@@ -1180,10 +1710,26 @@
       <c r="F35" s="5" t="n">
         <v>162.200424222168</v>
       </c>
+      <c r="G35" s="0"/>
+      <c r="H35" s="0"/>
+      <c r="I35" s="0"/>
+      <c r="J35" s="0"/>
+      <c r="L35" s="0"/>
+      <c r="M35" s="0"/>
+      <c r="N35" s="0"/>
+      <c r="O35" s="6"/>
+      <c r="P35" s="6"/>
+      <c r="Q35" s="6"/>
+      <c r="R35" s="6"/>
+      <c r="S35" s="6"/>
+      <c r="T35" s="6"/>
+      <c r="U35" s="6"/>
+      <c r="V35" s="6"/>
+      <c r="W35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>-7.744135</v>
@@ -1200,10 +1746,26 @@
       <c r="F36" s="5" t="n">
         <v>103.0586736521</v>
       </c>
+      <c r="G36" s="0"/>
+      <c r="H36" s="0"/>
+      <c r="I36" s="0"/>
+      <c r="J36" s="0"/>
+      <c r="L36" s="0"/>
+      <c r="M36" s="0"/>
+      <c r="N36" s="0"/>
+      <c r="O36" s="6"/>
+      <c r="P36" s="6"/>
+      <c r="Q36" s="6"/>
+      <c r="R36" s="6"/>
+      <c r="S36" s="6"/>
+      <c r="T36" s="6"/>
+      <c r="U36" s="6"/>
+      <c r="V36" s="6"/>
+      <c r="W36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>-7.747075</v>
@@ -1220,10 +1782,26 @@
       <c r="F37" s="5" t="n">
         <v>102.347770690918</v>
       </c>
+      <c r="G37" s="0"/>
+      <c r="H37" s="0"/>
+      <c r="I37" s="0"/>
+      <c r="J37" s="0"/>
+      <c r="L37" s="0"/>
+      <c r="M37" s="0"/>
+      <c r="N37" s="0"/>
+      <c r="O37" s="6"/>
+      <c r="P37" s="6"/>
+      <c r="Q37" s="6"/>
+      <c r="R37" s="6"/>
+      <c r="S37" s="6"/>
+      <c r="T37" s="6"/>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6"/>
+      <c r="W37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>-7.73901333333333</v>
@@ -1240,10 +1818,26 @@
       <c r="F38" s="5" t="n">
         <v>110.125648498535</v>
       </c>
+      <c r="G38" s="0"/>
+      <c r="H38" s="0"/>
+      <c r="I38" s="0"/>
+      <c r="J38" s="0"/>
+      <c r="L38" s="0"/>
+      <c r="M38" s="0"/>
+      <c r="N38" s="0"/>
+      <c r="O38" s="6"/>
+      <c r="P38" s="6"/>
+      <c r="Q38" s="6"/>
+      <c r="R38" s="6"/>
+      <c r="S38" s="6"/>
+      <c r="T38" s="6"/>
+      <c r="U38" s="6"/>
+      <c r="V38" s="6"/>
+      <c r="W38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>-7.73855333333333</v>
@@ -1260,10 +1854,26 @@
       <c r="F39" s="5" t="n">
         <v>114.826515197754</v>
       </c>
+      <c r="G39" s="0"/>
+      <c r="H39" s="0"/>
+      <c r="I39" s="0"/>
+      <c r="J39" s="0"/>
+      <c r="L39" s="0"/>
+      <c r="M39" s="0"/>
+      <c r="N39" s="0"/>
+      <c r="O39" s="6"/>
+      <c r="P39" s="6"/>
+      <c r="Q39" s="6"/>
+      <c r="R39" s="6"/>
+      <c r="S39" s="6"/>
+      <c r="T39" s="6"/>
+      <c r="U39" s="6"/>
+      <c r="V39" s="6"/>
+      <c r="W39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>-7.736845</v>
@@ -1280,10 +1890,26 @@
       <c r="F40" s="5" t="n">
         <v>113.601337464844</v>
       </c>
+      <c r="G40" s="0"/>
+      <c r="H40" s="0"/>
+      <c r="I40" s="0"/>
+      <c r="J40" s="0"/>
+      <c r="L40" s="0"/>
+      <c r="M40" s="0"/>
+      <c r="N40" s="0"/>
+      <c r="O40" s="6"/>
+      <c r="P40" s="6"/>
+      <c r="Q40" s="6"/>
+      <c r="R40" s="6"/>
+      <c r="S40" s="6"/>
+      <c r="T40" s="6"/>
+      <c r="U40" s="6"/>
+      <c r="V40" s="6"/>
+      <c r="W40" s="6"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>-7.730785</v>
@@ -1300,10 +1926,26 @@
       <c r="F41" s="5" t="n">
         <v>113.723861694336</v>
       </c>
+      <c r="G41" s="0"/>
+      <c r="H41" s="0"/>
+      <c r="I41" s="0"/>
+      <c r="J41" s="0"/>
+      <c r="L41" s="0"/>
+      <c r="M41" s="0"/>
+      <c r="N41" s="0"/>
+      <c r="O41" s="6"/>
+      <c r="P41" s="6"/>
+      <c r="Q41" s="6"/>
+      <c r="R41" s="6"/>
+      <c r="S41" s="6"/>
+      <c r="T41" s="6"/>
+      <c r="U41" s="6"/>
+      <c r="V41" s="6"/>
+      <c r="W41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>-7.73390833333333</v>
@@ -1320,10 +1962,26 @@
       <c r="F42" s="5" t="n">
         <v>118.082794189453</v>
       </c>
+      <c r="G42" s="0"/>
+      <c r="H42" s="0"/>
+      <c r="I42" s="0"/>
+      <c r="J42" s="0"/>
+      <c r="L42" s="0"/>
+      <c r="M42" s="0"/>
+      <c r="N42" s="0"/>
+      <c r="O42" s="6"/>
+      <c r="P42" s="6"/>
+      <c r="Q42" s="6"/>
+      <c r="R42" s="6"/>
+      <c r="S42" s="6"/>
+      <c r="T42" s="6"/>
+      <c r="U42" s="6"/>
+      <c r="V42" s="6"/>
+      <c r="W42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>-7.74343</v>
@@ -1340,10 +1998,26 @@
       <c r="F43" s="5" t="n">
         <v>117.907688356201</v>
       </c>
+      <c r="G43" s="0"/>
+      <c r="H43" s="0"/>
+      <c r="I43" s="0"/>
+      <c r="J43" s="0"/>
+      <c r="L43" s="0"/>
+      <c r="M43" s="0"/>
+      <c r="N43" s="0"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="6"/>
+      <c r="Q43" s="6"/>
+      <c r="R43" s="6"/>
+      <c r="S43" s="6"/>
+      <c r="T43" s="6"/>
+      <c r="U43" s="6"/>
+      <c r="V43" s="6"/>
+      <c r="W43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B44" s="3" t="n">
         <v>-7.74878666666667</v>
@@ -1360,10 +2034,26 @@
       <c r="F44" s="5" t="n">
         <v>96.8182830810547</v>
       </c>
+      <c r="G44" s="0"/>
+      <c r="H44" s="0"/>
+      <c r="I44" s="0"/>
+      <c r="J44" s="0"/>
+      <c r="L44" s="0"/>
+      <c r="M44" s="0"/>
+      <c r="N44" s="0"/>
+      <c r="O44" s="6"/>
+      <c r="P44" s="6"/>
+      <c r="Q44" s="6"/>
+      <c r="R44" s="6"/>
+      <c r="S44" s="6"/>
+      <c r="T44" s="6"/>
+      <c r="U44" s="6"/>
+      <c r="V44" s="6"/>
+      <c r="W44" s="6"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>-7.76058965774792</v>
@@ -1380,10 +2070,26 @@
       <c r="F45" s="5" t="n">
         <v>99.9816704658203</v>
       </c>
+      <c r="G45" s="0"/>
+      <c r="H45" s="0"/>
+      <c r="I45" s="0"/>
+      <c r="J45" s="0"/>
+      <c r="L45" s="0"/>
+      <c r="M45" s="0"/>
+      <c r="N45" s="0"/>
+      <c r="O45" s="6"/>
+      <c r="P45" s="6"/>
+      <c r="Q45" s="6"/>
+      <c r="R45" s="6"/>
+      <c r="S45" s="6"/>
+      <c r="T45" s="6"/>
+      <c r="U45" s="6"/>
+      <c r="V45" s="6"/>
+      <c r="W45" s="6"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B46" s="3" t="n">
         <v>-7.75120845129024</v>
@@ -1400,10 +2106,26 @@
       <c r="F46" s="5" t="n">
         <v>116.905540466309</v>
       </c>
+      <c r="G46" s="0"/>
+      <c r="H46" s="0"/>
+      <c r="I46" s="0"/>
+      <c r="J46" s="0"/>
+      <c r="L46" s="0"/>
+      <c r="M46" s="0"/>
+      <c r="N46" s="0"/>
+      <c r="O46" s="6"/>
+      <c r="P46" s="6"/>
+      <c r="Q46" s="6"/>
+      <c r="R46" s="6"/>
+      <c r="S46" s="6"/>
+      <c r="T46" s="6"/>
+      <c r="U46" s="6"/>
+      <c r="V46" s="6"/>
+      <c r="W46" s="6"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B47" s="3" t="n">
         <v>-7.746465</v>
@@ -1420,10 +2142,26 @@
       <c r="F47" s="5" t="n">
         <v>110.521766662598</v>
       </c>
+      <c r="G47" s="0"/>
+      <c r="H47" s="0"/>
+      <c r="I47" s="0"/>
+      <c r="J47" s="0"/>
+      <c r="L47" s="0"/>
+      <c r="M47" s="0"/>
+      <c r="N47" s="0"/>
+      <c r="O47" s="6"/>
+      <c r="P47" s="6"/>
+      <c r="Q47" s="6"/>
+      <c r="R47" s="6"/>
+      <c r="S47" s="6"/>
+      <c r="T47" s="6"/>
+      <c r="U47" s="6"/>
+      <c r="V47" s="6"/>
+      <c r="W47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B48" s="3" t="n">
         <v>-7.73529666666667</v>
@@ -1440,10 +2178,26 @@
       <c r="F48" s="5" t="n">
         <v>119.422584693359</v>
       </c>
+      <c r="G48" s="0"/>
+      <c r="H48" s="0"/>
+      <c r="I48" s="0"/>
+      <c r="J48" s="0"/>
+      <c r="L48" s="0"/>
+      <c r="M48" s="0"/>
+      <c r="N48" s="0"/>
+      <c r="O48" s="6"/>
+      <c r="P48" s="6"/>
+      <c r="Q48" s="6"/>
+      <c r="R48" s="6"/>
+      <c r="S48" s="6"/>
+      <c r="T48" s="6"/>
+      <c r="U48" s="6"/>
+      <c r="V48" s="6"/>
+      <c r="W48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B49" s="3" t="n">
         <v>-7.73211166666667</v>
@@ -1460,10 +2214,26 @@
       <c r="F49" s="5" t="n">
         <v>129.631423950195</v>
       </c>
+      <c r="G49" s="0"/>
+      <c r="H49" s="0"/>
+      <c r="I49" s="0"/>
+      <c r="J49" s="0"/>
+      <c r="L49" s="0"/>
+      <c r="M49" s="0"/>
+      <c r="N49" s="0"/>
+      <c r="O49" s="6"/>
+      <c r="P49" s="6"/>
+      <c r="Q49" s="6"/>
+      <c r="R49" s="6"/>
+      <c r="S49" s="6"/>
+      <c r="T49" s="6"/>
+      <c r="U49" s="6"/>
+      <c r="V49" s="6"/>
+      <c r="W49" s="6"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B50" s="3" t="n">
         <v>-7.74282666666667</v>
@@ -1480,10 +2250,26 @@
       <c r="F50" s="5" t="n">
         <v>123.278053337646</v>
       </c>
+      <c r="G50" s="0"/>
+      <c r="H50" s="0"/>
+      <c r="I50" s="0"/>
+      <c r="J50" s="0"/>
+      <c r="L50" s="0"/>
+      <c r="M50" s="0"/>
+      <c r="N50" s="0"/>
+      <c r="O50" s="6"/>
+      <c r="P50" s="6"/>
+      <c r="Q50" s="6"/>
+      <c r="R50" s="6"/>
+      <c r="S50" s="6"/>
+      <c r="T50" s="6"/>
+      <c r="U50" s="6"/>
+      <c r="V50" s="6"/>
+      <c r="W50" s="6"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B51" s="3" t="n">
         <v>-7.75552289561845</v>
@@ -1500,10 +2286,26 @@
       <c r="F51" s="5" t="n">
         <v>108.985710144043</v>
       </c>
+      <c r="G51" s="0"/>
+      <c r="H51" s="0"/>
+      <c r="I51" s="0"/>
+      <c r="J51" s="0"/>
+      <c r="L51" s="0"/>
+      <c r="M51" s="0"/>
+      <c r="N51" s="0"/>
+      <c r="O51" s="6"/>
+      <c r="P51" s="6"/>
+      <c r="Q51" s="6"/>
+      <c r="R51" s="6"/>
+      <c r="S51" s="6"/>
+      <c r="T51" s="6"/>
+      <c r="U51" s="6"/>
+      <c r="V51" s="6"/>
+      <c r="W51" s="6"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B52" s="3" t="n">
         <v>-7.76307666666667</v>
@@ -1520,10 +2322,26 @@
       <c r="F52" s="5" t="n">
         <v>109.82119761499</v>
       </c>
+      <c r="G52" s="0"/>
+      <c r="H52" s="0"/>
+      <c r="I52" s="0"/>
+      <c r="J52" s="0"/>
+      <c r="L52" s="0"/>
+      <c r="M52" s="0"/>
+      <c r="N52" s="0"/>
+      <c r="O52" s="6"/>
+      <c r="P52" s="6"/>
+      <c r="Q52" s="6"/>
+      <c r="R52" s="6"/>
+      <c r="S52" s="6"/>
+      <c r="T52" s="6"/>
+      <c r="U52" s="6"/>
+      <c r="V52" s="6"/>
+      <c r="W52" s="6"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B53" s="3" t="n">
         <v>-7.720965</v>
@@ -1540,10 +2358,26 @@
       <c r="F53" s="5" t="n">
         <v>167.074172973633</v>
       </c>
+      <c r="G53" s="0"/>
+      <c r="H53" s="0"/>
+      <c r="I53" s="0"/>
+      <c r="J53" s="0"/>
+      <c r="L53" s="0"/>
+      <c r="M53" s="0"/>
+      <c r="N53" s="0"/>
+      <c r="O53" s="6"/>
+      <c r="P53" s="6"/>
+      <c r="Q53" s="6"/>
+      <c r="R53" s="6"/>
+      <c r="S53" s="6"/>
+      <c r="T53" s="6"/>
+      <c r="U53" s="6"/>
+      <c r="V53" s="6"/>
+      <c r="W53" s="6"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B54" s="3" t="n">
         <v>-7.72067601534982</v>
@@ -1560,10 +2394,26 @@
       <c r="F54" s="5" t="n">
         <v>216.702954231122</v>
       </c>
+      <c r="G54" s="0"/>
+      <c r="H54" s="0"/>
+      <c r="I54" s="0"/>
+      <c r="J54" s="0"/>
+      <c r="L54" s="0"/>
+      <c r="M54" s="0"/>
+      <c r="N54" s="0"/>
+      <c r="O54" s="6"/>
+      <c r="P54" s="6"/>
+      <c r="Q54" s="6"/>
+      <c r="R54" s="6"/>
+      <c r="S54" s="6"/>
+      <c r="T54" s="6"/>
+      <c r="U54" s="6"/>
+      <c r="V54" s="6"/>
+      <c r="W54" s="6"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B55" s="3" t="n">
         <v>-7.71763077414723</v>
@@ -1580,10 +2430,26 @@
       <c r="F55" s="5" t="n">
         <v>357.373662546629</v>
       </c>
+      <c r="G55" s="0"/>
+      <c r="H55" s="0"/>
+      <c r="I55" s="0"/>
+      <c r="J55" s="0"/>
+      <c r="L55" s="0"/>
+      <c r="M55" s="0"/>
+      <c r="N55" s="0"/>
+      <c r="O55" s="6"/>
+      <c r="P55" s="6"/>
+      <c r="Q55" s="6"/>
+      <c r="R55" s="6"/>
+      <c r="S55" s="6"/>
+      <c r="T55" s="6"/>
+      <c r="U55" s="6"/>
+      <c r="V55" s="6"/>
+      <c r="W55" s="6"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B56" s="3" t="n">
         <v>-7.7161896198009</v>
@@ -1600,10 +2466,26 @@
       <c r="F56" s="5" t="n">
         <v>132.581039268066</v>
       </c>
+      <c r="G56" s="0"/>
+      <c r="H56" s="0"/>
+      <c r="I56" s="0"/>
+      <c r="J56" s="0"/>
+      <c r="L56" s="0"/>
+      <c r="M56" s="0"/>
+      <c r="N56" s="0"/>
+      <c r="O56" s="6"/>
+      <c r="P56" s="6"/>
+      <c r="Q56" s="6"/>
+      <c r="R56" s="6"/>
+      <c r="S56" s="6"/>
+      <c r="T56" s="6"/>
+      <c r="U56" s="6"/>
+      <c r="V56" s="6"/>
+      <c r="W56" s="6"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B57" s="3" t="n">
         <v>-7.7136595</v>
@@ -1620,11 +2502,26 @@
       <c r="F57" s="5" t="n">
         <v>263.128784376953</v>
       </c>
-      <c r="G57" s="6"/>
+      <c r="G57" s="0"/>
+      <c r="H57" s="0"/>
+      <c r="I57" s="0"/>
+      <c r="J57" s="0"/>
+      <c r="L57" s="0"/>
+      <c r="M57" s="0"/>
+      <c r="N57" s="0"/>
+      <c r="O57" s="6"/>
+      <c r="P57" s="6"/>
+      <c r="Q57" s="6"/>
+      <c r="R57" s="6"/>
+      <c r="S57" s="6"/>
+      <c r="T57" s="6"/>
+      <c r="U57" s="6"/>
+      <c r="V57" s="6"/>
+      <c r="W57" s="6"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B58" s="3" t="n">
         <v>-7.710344</v>
@@ -1641,10 +2538,26 @@
       <c r="F58" s="5" t="n">
         <v>386.825546503906</v>
       </c>
+      <c r="G58" s="0"/>
+      <c r="H58" s="0"/>
+      <c r="I58" s="0"/>
+      <c r="J58" s="0"/>
+      <c r="L58" s="0"/>
+      <c r="M58" s="0"/>
+      <c r="N58" s="0"/>
+      <c r="O58" s="6"/>
+      <c r="P58" s="6"/>
+      <c r="Q58" s="6"/>
+      <c r="R58" s="6"/>
+      <c r="S58" s="6"/>
+      <c r="T58" s="6"/>
+      <c r="U58" s="6"/>
+      <c r="V58" s="6"/>
+      <c r="W58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B59" s="3" t="n">
         <v>-7.71324527</v>
@@ -1661,10 +2574,26 @@
       <c r="F59" s="5" t="n">
         <v>390.998794449219</v>
       </c>
+      <c r="G59" s="0"/>
+      <c r="H59" s="0"/>
+      <c r="I59" s="0"/>
+      <c r="J59" s="0"/>
+      <c r="L59" s="0"/>
+      <c r="M59" s="0"/>
+      <c r="N59" s="0"/>
+      <c r="O59" s="6"/>
+      <c r="P59" s="6"/>
+      <c r="Q59" s="6"/>
+      <c r="R59" s="6"/>
+      <c r="S59" s="6"/>
+      <c r="T59" s="6"/>
+      <c r="U59" s="6"/>
+      <c r="V59" s="6"/>
+      <c r="W59" s="6"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B60" s="3" t="n">
         <v>-7.7193371</v>
@@ -1681,10 +2610,26 @@
       <c r="F60" s="5" t="n">
         <v>431.893676511719</v>
       </c>
+      <c r="G60" s="0"/>
+      <c r="H60" s="0"/>
+      <c r="I60" s="0"/>
+      <c r="J60" s="0"/>
+      <c r="L60" s="0"/>
+      <c r="M60" s="0"/>
+      <c r="N60" s="0"/>
+      <c r="O60" s="6"/>
+      <c r="P60" s="6"/>
+      <c r="Q60" s="6"/>
+      <c r="R60" s="6"/>
+      <c r="S60" s="6"/>
+      <c r="T60" s="6"/>
+      <c r="U60" s="6"/>
+      <c r="V60" s="6"/>
+      <c r="W60" s="6"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B61" s="3" t="n">
         <v>-7.724188431</v>
@@ -1701,6 +2646,22 @@
       <c r="F61" s="5" t="n">
         <v>314.894424208008</v>
       </c>
+      <c r="G61" s="0"/>
+      <c r="H61" s="0"/>
+      <c r="I61" s="0"/>
+      <c r="J61" s="0"/>
+      <c r="L61" s="0"/>
+      <c r="M61" s="0"/>
+      <c r="N61" s="0"/>
+      <c r="O61" s="6"/>
+      <c r="P61" s="6"/>
+      <c r="Q61" s="6"/>
+      <c r="R61" s="6"/>
+      <c r="S61" s="6"/>
+      <c r="T61" s="6"/>
+      <c r="U61" s="6"/>
+      <c r="V61" s="6"/>
+      <c r="W61" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Update plot data sheet
</commit_message>
<xml_diff>
--- a/passive_seismic/plot_data.xlsx
+++ b/passive_seismic/plot_data.xlsx
@@ -25,22 +25,22 @@
     <t xml:space="preserve">STATION</t>
   </si>
   <si>
+    <t xml:space="preserve">LONGITUDE</t>
+  </si>
+  <si>
     <t xml:space="preserve">LATITUDE</t>
   </si>
   <si>
-    <t xml:space="preserve">LONGITUDE</t>
+    <t xml:space="preserve">EASTING</t>
   </si>
   <si>
     <t xml:space="preserve">NORTHING</t>
   </si>
   <si>
-    <t xml:space="preserve">EASTING</t>
-  </si>
-  <si>
     <t xml:space="preserve">ELEVATION</t>
   </si>
   <si>
-    <t xml:space="preserve">f0 (Hz)</t>
+    <t xml:space="preserve">f0</t>
   </si>
   <si>
     <t xml:space="preserve">A0</t>
@@ -463,10 +463,8 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="13.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="11.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.73"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="11.53"/>
   </cols>
@@ -502,33 +500,32 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="3" t="n">
+        <v>110.1809619169</v>
+      </c>
+      <c r="C2" s="3" t="n">
         <v>-7.74603882435985</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>110.1809619169</v>
-      </c>
       <c r="D2" s="4" t="n">
+        <v>9143690.77372846</v>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>409684.71005509</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>9143690.77372846</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>191.163032529785</v>
       </c>
-      <c r="G2" s="0"/>
-      <c r="H2" s="0"/>
-      <c r="I2" s="0"/>
-      <c r="J2" s="0"/>
-      <c r="L2" s="0"/>
-      <c r="M2" s="0"/>
-      <c r="N2" s="0"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="0"/>
       <c r="O2" s="6"/>
       <c r="P2" s="6"/>
       <c r="Q2" s="6"/>
@@ -544,27 +541,25 @@
         <v>11</v>
       </c>
       <c r="B3" s="3" t="n">
+        <v>110.189506530762</v>
+      </c>
+      <c r="C3" s="3" t="n">
         <v>-7.74663162231445</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>110.189506530762</v>
-      </c>
       <c r="D3" s="4" t="n">
+        <v>9143627.03956445</v>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>410627.110483121</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>9143627.03956445</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>185.148940991211</v>
       </c>
-      <c r="G3" s="0"/>
-      <c r="H3" s="0"/>
-      <c r="I3" s="0"/>
-      <c r="J3" s="0"/>
-      <c r="L3" s="0"/>
-      <c r="M3" s="0"/>
-      <c r="N3" s="0"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="0"/>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="6"/>
@@ -580,27 +575,25 @@
         <v>12</v>
       </c>
       <c r="B4" s="3" t="n">
+        <v>110.195628333333</v>
+      </c>
+      <c r="C4" s="3" t="n">
         <v>-7.75365666666666</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>110.195628333333</v>
-      </c>
       <c r="D4" s="4" t="n">
+        <v>9142851.62748084</v>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>411303.673677725</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>9142851.62748084</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>127.667381254395</v>
       </c>
-      <c r="G4" s="0"/>
-      <c r="H4" s="0"/>
-      <c r="I4" s="0"/>
-      <c r="J4" s="0"/>
-      <c r="L4" s="0"/>
-      <c r="M4" s="0"/>
-      <c r="N4" s="0"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="0"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
@@ -616,27 +609,25 @@
         <v>13</v>
       </c>
       <c r="B5" s="3" t="n">
+        <v>110.199602180347</v>
+      </c>
+      <c r="C5" s="3" t="n">
         <v>-7.75709405564505</v>
       </c>
-      <c r="C5" s="3" t="n">
-        <v>110.199602180347</v>
-      </c>
       <c r="D5" s="4" t="n">
+        <v>9142472.41527113</v>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>411742.605391454</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>9142472.41527113</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>104.056293674316</v>
       </c>
-      <c r="G5" s="0"/>
-      <c r="H5" s="0"/>
-      <c r="I5" s="0"/>
-      <c r="J5" s="0"/>
-      <c r="L5" s="0"/>
-      <c r="M5" s="0"/>
-      <c r="N5" s="0"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="0"/>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
@@ -652,27 +643,25 @@
         <v>14</v>
       </c>
       <c r="B6" s="3" t="n">
+        <v>110.20624</v>
+      </c>
+      <c r="C6" s="3" t="n">
         <v>-7.76309333333333</v>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>110.20624</v>
-      </c>
       <c r="D6" s="4" t="n">
+        <v>9141810.50620388</v>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>412475.823695373</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>9141810.50620388</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>97.0373458862305</v>
       </c>
-      <c r="G6" s="0"/>
-      <c r="H6" s="0"/>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-      <c r="L6" s="0"/>
-      <c r="M6" s="0"/>
-      <c r="N6" s="0"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="0"/>
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
@@ -688,27 +677,25 @@
         <v>15</v>
       </c>
       <c r="B7" s="3" t="n">
+        <v>110.182843060258</v>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>-7.73740890654394</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>110.182843060258</v>
-      </c>
       <c r="D7" s="4" t="n">
+        <v>9144645.3061774</v>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>409890.324083769</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>9144645.3061774</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>347.634552001953</v>
       </c>
-      <c r="G7" s="0"/>
-      <c r="H7" s="0"/>
-      <c r="I7" s="0"/>
-      <c r="J7" s="0"/>
-      <c r="L7" s="0"/>
-      <c r="M7" s="0"/>
-      <c r="N7" s="0"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="0"/>
       <c r="O7" s="6"/>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
@@ -724,27 +711,25 @@
         <v>16</v>
       </c>
       <c r="B8" s="3" t="n">
+        <v>110.186089</v>
+      </c>
+      <c r="C8" s="3" t="n">
         <v>-7.738853</v>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>110.186089</v>
-      </c>
       <c r="D8" s="4" t="n">
+        <v>9144486.33178886</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>410248.589741817</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>9144486.33178886</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>216.977668832031</v>
       </c>
-      <c r="G8" s="0"/>
-      <c r="H8" s="0"/>
-      <c r="I8" s="0"/>
-      <c r="J8" s="0"/>
-      <c r="L8" s="0"/>
-      <c r="M8" s="0"/>
-      <c r="N8" s="0"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="0"/>
       <c r="O8" s="6"/>
       <c r="P8" s="6"/>
       <c r="Q8" s="6"/>
@@ -760,27 +745,25 @@
         <v>17</v>
       </c>
       <c r="B9" s="3" t="n">
+        <v>110.19143</v>
+      </c>
+      <c r="C9" s="3" t="n">
         <v>-7.743</v>
       </c>
-      <c r="C9" s="3" t="n">
-        <v>110.19143</v>
-      </c>
       <c r="D9" s="4" t="n">
+        <v>9144028.95893974</v>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>410838.460933084</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>9144028.95893974</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>172.269851465332</v>
       </c>
-      <c r="G9" s="0"/>
-      <c r="H9" s="0"/>
-      <c r="I9" s="0"/>
-      <c r="J9" s="0"/>
-      <c r="L9" s="0"/>
-      <c r="M9" s="0"/>
-      <c r="N9" s="0"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="0"/>
       <c r="O9" s="6"/>
       <c r="P9" s="6"/>
       <c r="Q9" s="6"/>
@@ -796,27 +779,25 @@
         <v>18</v>
       </c>
       <c r="B10" s="3" t="n">
+        <v>110.197905</v>
+      </c>
+      <c r="C10" s="3" t="n">
         <v>-7.743479</v>
       </c>
-      <c r="C10" s="3" t="n">
-        <v>110.197905</v>
-      </c>
       <c r="D10" s="4" t="n">
+        <v>9143977.35265984</v>
+      </c>
+      <c r="E10" s="4" t="n">
         <v>411552.608721983</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>9143977.35265984</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>112.366561804688</v>
       </c>
-      <c r="G10" s="0"/>
-      <c r="H10" s="0"/>
-      <c r="I10" s="0"/>
-      <c r="J10" s="0"/>
-      <c r="L10" s="0"/>
-      <c r="M10" s="0"/>
-      <c r="N10" s="0"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="0"/>
       <c r="O10" s="6"/>
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
@@ -832,27 +813,25 @@
         <v>19</v>
       </c>
       <c r="B11" s="3" t="n">
+        <v>110.206152402145</v>
+      </c>
+      <c r="C11" s="3" t="n">
         <v>-7.74505401956837</v>
       </c>
-      <c r="C11" s="3" t="n">
-        <v>110.206152402145</v>
-      </c>
       <c r="D11" s="4" t="n">
+        <v>9143804.92453015</v>
+      </c>
+      <c r="E11" s="4" t="n">
         <v>412462.435510075</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>9143804.92453015</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>111.736358530518</v>
       </c>
-      <c r="G11" s="0"/>
-      <c r="H11" s="0"/>
-      <c r="I11" s="0"/>
-      <c r="J11" s="0"/>
-      <c r="L11" s="0"/>
-      <c r="M11" s="0"/>
-      <c r="N11" s="0"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="0"/>
       <c r="O11" s="6"/>
       <c r="P11" s="6"/>
       <c r="Q11" s="6"/>
@@ -868,27 +847,25 @@
         <v>20</v>
       </c>
       <c r="B12" s="3" t="n">
+        <v>110.211748333333</v>
+      </c>
+      <c r="C12" s="3" t="n">
         <v>-7.74790333333333</v>
       </c>
-      <c r="C12" s="3" t="n">
-        <v>110.211748333333</v>
-      </c>
       <c r="D12" s="4" t="n">
+        <v>9143491.05163186</v>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>413080.120884984</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>9143491.05163186</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>99.3031997680664</v>
       </c>
-      <c r="G12" s="0"/>
-      <c r="H12" s="0"/>
-      <c r="I12" s="0"/>
-      <c r="J12" s="0"/>
-      <c r="L12" s="0"/>
-      <c r="M12" s="0"/>
-      <c r="N12" s="0"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="0"/>
       <c r="O12" s="6"/>
       <c r="P12" s="6"/>
       <c r="Q12" s="6"/>
@@ -904,27 +881,25 @@
         <v>21</v>
       </c>
       <c r="B13" s="3" t="n">
+        <v>110.188398333333</v>
+      </c>
+      <c r="C13" s="3" t="n">
         <v>-7.731415</v>
       </c>
-      <c r="C13" s="3" t="n">
-        <v>110.188398333333</v>
-      </c>
       <c r="D13" s="4" t="n">
+        <v>9145309.1703852</v>
+      </c>
+      <c r="E13" s="4" t="n">
         <v>410501.692623608</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>9145309.1703852</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>282.519851674805</v>
       </c>
-      <c r="G13" s="0"/>
-      <c r="H13" s="0"/>
-      <c r="I13" s="0"/>
-      <c r="J13" s="0"/>
-      <c r="L13" s="0"/>
-      <c r="M13" s="0"/>
-      <c r="N13" s="0"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="0"/>
       <c r="O13" s="6"/>
       <c r="P13" s="6"/>
       <c r="Q13" s="6"/>
@@ -940,27 +915,25 @@
         <v>22</v>
       </c>
       <c r="B14" s="3" t="n">
+        <v>110.197805</v>
+      </c>
+      <c r="C14" s="3" t="n">
         <v>-7.73346</v>
       </c>
-      <c r="C14" s="3" t="n">
-        <v>110.197805</v>
-      </c>
       <c r="D14" s="4" t="n">
+        <v>9145085.03936802</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>411539.492533147</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>9145085.03936802</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>122.482795642578</v>
       </c>
-      <c r="G14" s="0"/>
-      <c r="H14" s="0"/>
-      <c r="I14" s="0"/>
-      <c r="J14" s="0"/>
-      <c r="L14" s="0"/>
-      <c r="M14" s="0"/>
-      <c r="N14" s="0"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="0"/>
       <c r="O14" s="6"/>
       <c r="P14" s="6"/>
       <c r="Q14" s="6"/>
@@ -976,27 +949,25 @@
         <v>23</v>
       </c>
       <c r="B15" s="3" t="n">
+        <v>110.205475</v>
+      </c>
+      <c r="C15" s="3" t="n">
         <v>-7.73511</v>
       </c>
-      <c r="C15" s="3" t="n">
-        <v>110.205475</v>
-      </c>
       <c r="D15" s="4" t="n">
+        <v>9144904.20069305</v>
+      </c>
+      <c r="E15" s="4" t="n">
         <v>412385.680327005</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>9144904.20069305</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>112.215297560547</v>
       </c>
-      <c r="G15" s="0"/>
-      <c r="H15" s="0"/>
-      <c r="I15" s="0"/>
-      <c r="J15" s="0"/>
-      <c r="L15" s="0"/>
-      <c r="M15" s="0"/>
-      <c r="N15" s="0"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="0"/>
       <c r="O15" s="6"/>
       <c r="P15" s="6"/>
       <c r="Q15" s="6"/>
@@ -1012,27 +983,25 @@
         <v>24</v>
       </c>
       <c r="B16" s="3" t="n">
+        <v>110.210888333333</v>
+      </c>
+      <c r="C16" s="3" t="n">
         <v>-7.73861166666666</v>
       </c>
-      <c r="C16" s="3" t="n">
-        <v>110.210888333333</v>
-      </c>
       <c r="D16" s="4" t="n">
+        <v>9144518.16573203</v>
+      </c>
+      <c r="E16" s="4" t="n">
         <v>412983.377155415</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>9144518.16573203</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>105.960304286133</v>
       </c>
-      <c r="G16" s="0"/>
-      <c r="H16" s="0"/>
-      <c r="I16" s="0"/>
-      <c r="J16" s="0"/>
-      <c r="L16" s="0"/>
-      <c r="M16" s="0"/>
-      <c r="N16" s="0"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="0"/>
       <c r="O16" s="6"/>
       <c r="P16" s="6"/>
       <c r="Q16" s="6"/>
@@ -1048,27 +1017,25 @@
         <v>25</v>
       </c>
       <c r="B17" s="3" t="n">
+        <v>110.218589457321</v>
+      </c>
+      <c r="C17" s="3" t="n">
         <v>-7.74097385669832</v>
       </c>
-      <c r="C17" s="3" t="n">
-        <v>110.218589457321</v>
-      </c>
       <c r="D17" s="4" t="n">
+        <v>9144258.56904513</v>
+      </c>
+      <c r="E17" s="4" t="n">
         <v>413833.123636272</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>9144258.56904513</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>101.337562561035</v>
       </c>
-      <c r="G17" s="0"/>
-      <c r="H17" s="0"/>
-      <c r="I17" s="0"/>
-      <c r="J17" s="0"/>
-      <c r="L17" s="0"/>
-      <c r="M17" s="0"/>
-      <c r="N17" s="0"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="0"/>
       <c r="O17" s="6"/>
       <c r="P17" s="6"/>
       <c r="Q17" s="6"/>
@@ -1084,27 +1051,25 @@
         <v>26</v>
       </c>
       <c r="B18" s="3" t="n">
+        <v>110.197053333333</v>
+      </c>
+      <c r="C18" s="3" t="n">
         <v>-7.72301666666666</v>
       </c>
-      <c r="C18" s="3" t="n">
-        <v>110.197053333333</v>
-      </c>
       <c r="D18" s="4" t="n">
+        <v>9146239.50487017</v>
+      </c>
+      <c r="E18" s="4" t="n">
         <v>411454.422606736</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>9146239.50487017</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>197.519668579102</v>
       </c>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0"/>
-      <c r="I18" s="0"/>
-      <c r="J18" s="0"/>
-      <c r="L18" s="0"/>
-      <c r="M18" s="0"/>
-      <c r="N18" s="0"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="0"/>
       <c r="O18" s="6"/>
       <c r="P18" s="6"/>
       <c r="Q18" s="6"/>
@@ -1120,27 +1085,25 @@
         <v>27</v>
       </c>
       <c r="B19" s="3" t="n">
+        <v>110.20297</v>
+      </c>
+      <c r="C19" s="3" t="n">
         <v>-7.725055</v>
       </c>
-      <c r="C19" s="3" t="n">
-        <v>110.20297</v>
-      </c>
       <c r="D19" s="4" t="n">
+        <v>9146015.37016071</v>
+      </c>
+      <c r="E19" s="4" t="n">
         <v>412107.350054431</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>9146015.37016071</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>142.18503559668</v>
       </c>
-      <c r="G19" s="0"/>
-      <c r="H19" s="0"/>
-      <c r="I19" s="0"/>
-      <c r="J19" s="0"/>
-      <c r="L19" s="0"/>
-      <c r="M19" s="0"/>
-      <c r="N19" s="0"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="0"/>
       <c r="O19" s="6"/>
       <c r="P19" s="6"/>
       <c r="Q19" s="6"/>
@@ -1156,27 +1119,25 @@
         <v>28</v>
       </c>
       <c r="B20" s="3" t="n">
+        <v>110.208996666667</v>
+      </c>
+      <c r="C20" s="3" t="n">
         <v>-7.72724666666667</v>
       </c>
-      <c r="C20" s="3" t="n">
-        <v>110.208996666667</v>
-      </c>
       <c r="D20" s="4" t="n">
+        <v>9145774.29693356</v>
+      </c>
+      <c r="E20" s="4" t="n">
         <v>412772.43287169</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>9145774.29693356</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>116.86959079248</v>
       </c>
-      <c r="G20" s="0"/>
-      <c r="H20" s="0"/>
-      <c r="I20" s="0"/>
-      <c r="J20" s="0"/>
-      <c r="L20" s="0"/>
-      <c r="M20" s="0"/>
-      <c r="N20" s="0"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="0"/>
       <c r="O20" s="6"/>
       <c r="P20" s="6"/>
       <c r="Q20" s="6"/>
@@ -1192,27 +1153,25 @@
         <v>29</v>
       </c>
       <c r="B21" s="3" t="n">
+        <v>110.214976666667</v>
+      </c>
+      <c r="C21" s="3" t="n">
         <v>-7.73107</v>
       </c>
-      <c r="C21" s="3" t="n">
-        <v>110.214976666667</v>
-      </c>
       <c r="D21" s="4" t="n">
+        <v>9145352.80808655</v>
+      </c>
+      <c r="E21" s="4" t="n">
         <v>413432.69407556</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>9145352.80808655</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>108.508556337646</v>
       </c>
-      <c r="G21" s="0"/>
-      <c r="H21" s="0"/>
-      <c r="I21" s="0"/>
-      <c r="J21" s="0"/>
-      <c r="L21" s="0"/>
-      <c r="M21" s="0"/>
-      <c r="N21" s="0"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="0"/>
       <c r="O21" s="6"/>
       <c r="P21" s="6"/>
       <c r="Q21" s="6"/>
@@ -1228,27 +1187,25 @@
         <v>30</v>
       </c>
       <c r="B22" s="3" t="n">
+        <v>110.220011666667</v>
+      </c>
+      <c r="C22" s="3" t="n">
         <v>-7.73054166666666</v>
       </c>
-      <c r="C22" s="3" t="n">
-        <v>110.220011666667</v>
-      </c>
       <c r="D22" s="4" t="n">
+        <v>9145412.24086345</v>
+      </c>
+      <c r="E22" s="4" t="n">
         <v>413987.847789588</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>9145412.24086345</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>95.2035522460938</v>
       </c>
-      <c r="G22" s="0"/>
-      <c r="H22" s="0"/>
-      <c r="I22" s="0"/>
-      <c r="J22" s="0"/>
-      <c r="L22" s="0"/>
-      <c r="M22" s="0"/>
-      <c r="N22" s="0"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="0"/>
       <c r="O22" s="6"/>
       <c r="P22" s="6"/>
       <c r="Q22" s="6"/>
@@ -1264,27 +1221,25 @@
         <v>31</v>
       </c>
       <c r="B23" s="3" t="n">
+        <v>110.205256955259</v>
+      </c>
+      <c r="C23" s="3" t="n">
         <v>-7.73295791631359</v>
       </c>
-      <c r="C23" s="3" t="n">
-        <v>110.205256955259</v>
-      </c>
       <c r="D23" s="4" t="n">
+        <v>9145142.09118594</v>
+      </c>
+      <c r="E23" s="4" t="n">
         <v>412361.190299079</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>9145142.09118594</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>113.839790344238</v>
       </c>
-      <c r="G23" s="0"/>
-      <c r="H23" s="0"/>
-      <c r="I23" s="0"/>
-      <c r="J23" s="0"/>
-      <c r="L23" s="0"/>
-      <c r="M23" s="0"/>
-      <c r="N23" s="0"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="0"/>
       <c r="O23" s="6"/>
       <c r="P23" s="6"/>
       <c r="Q23" s="6"/>
@@ -1300,27 +1255,25 @@
         <v>32</v>
       </c>
       <c r="B24" s="3" t="n">
+        <v>110.200280228297</v>
+      </c>
+      <c r="C24" s="3" t="n">
         <v>-7.72960051265161</v>
       </c>
-      <c r="C24" s="3" t="n">
-        <v>110.200280228297</v>
-      </c>
       <c r="D24" s="4" t="n">
+        <v>9145512.26007277</v>
+      </c>
+      <c r="E24" s="4" t="n">
         <v>411811.659483888</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>9145512.26007277</v>
       </c>
       <c r="F24" s="5" t="n">
         <v>136.683654851074</v>
       </c>
-      <c r="G24" s="0"/>
-      <c r="H24" s="0"/>
-      <c r="I24" s="0"/>
-      <c r="J24" s="0"/>
-      <c r="L24" s="0"/>
-      <c r="M24" s="0"/>
-      <c r="N24" s="0"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="0"/>
       <c r="O24" s="6"/>
       <c r="P24" s="6"/>
       <c r="Q24" s="6"/>
@@ -1336,27 +1289,25 @@
         <v>33</v>
       </c>
       <c r="B25" s="3" t="n">
+        <v>110.196628333333</v>
+      </c>
+      <c r="C25" s="3" t="n">
         <v>-7.74705</v>
       </c>
-      <c r="C25" s="3" t="n">
-        <v>110.196628333333</v>
-      </c>
       <c r="D25" s="4" t="n">
+        <v>9143582.27443123</v>
+      </c>
+      <c r="E25" s="4" t="n">
         <v>411412.567258259</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>9143582.27443123</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>106.308010254883</v>
       </c>
-      <c r="G25" s="0"/>
-      <c r="H25" s="0"/>
-      <c r="I25" s="0"/>
-      <c r="J25" s="0"/>
-      <c r="L25" s="0"/>
-      <c r="M25" s="0"/>
-      <c r="N25" s="0"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="0"/>
       <c r="O25" s="6"/>
       <c r="P25" s="6"/>
       <c r="Q25" s="6"/>
@@ -1372,27 +1323,25 @@
         <v>34</v>
       </c>
       <c r="B26" s="3" t="n">
+        <v>110.206350684013</v>
+      </c>
+      <c r="C26" s="3" t="n">
         <v>-7.74886467967605</v>
       </c>
-      <c r="C26" s="3" t="n">
-        <v>110.206350684013</v>
-      </c>
       <c r="D26" s="4" t="n">
+        <v>9143383.65684573</v>
+      </c>
+      <c r="E26" s="4" t="n">
         <v>412485.08812415</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>9143383.65684573</v>
       </c>
       <c r="F26" s="5" t="n">
         <v>103.607296213867</v>
       </c>
-      <c r="G26" s="0"/>
-      <c r="H26" s="0"/>
-      <c r="I26" s="0"/>
-      <c r="J26" s="0"/>
-      <c r="L26" s="0"/>
-      <c r="M26" s="0"/>
-      <c r="N26" s="0"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="0"/>
       <c r="O26" s="6"/>
       <c r="P26" s="6"/>
       <c r="Q26" s="6"/>
@@ -1408,27 +1357,25 @@
         <v>35</v>
       </c>
       <c r="B27" s="3" t="n">
+        <v>110.20786</v>
+      </c>
+      <c r="C27" s="3" t="n">
         <v>-7.75520166666667</v>
       </c>
-      <c r="C27" s="3" t="n">
-        <v>110.20786</v>
-      </c>
       <c r="D27" s="4" t="n">
+        <v>9142683.34702022</v>
+      </c>
+      <c r="E27" s="4" t="n">
         <v>412652.835822452</v>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>9142683.34702022</v>
       </c>
       <c r="F27" s="5" t="n">
         <v>105.647788823486</v>
       </c>
-      <c r="G27" s="0"/>
-      <c r="H27" s="0"/>
-      <c r="I27" s="0"/>
-      <c r="J27" s="0"/>
-      <c r="L27" s="0"/>
-      <c r="M27" s="0"/>
-      <c r="N27" s="0"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="0"/>
       <c r="O27" s="6"/>
       <c r="P27" s="6"/>
       <c r="Q27" s="6"/>
@@ -1444,27 +1391,25 @@
         <v>36</v>
       </c>
       <c r="B28" s="3" t="n">
+        <v>110.214983333333</v>
+      </c>
+      <c r="C28" s="3" t="n">
         <v>-7.751647823625</v>
       </c>
-      <c r="C28" s="3" t="n">
-        <v>110.214983333333</v>
-      </c>
       <c r="D28" s="4" t="n">
+        <v>9143077.72001354</v>
+      </c>
+      <c r="E28" s="4" t="n">
         <v>413437.62836366</v>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>9143077.72001354</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>104.428081663086</v>
       </c>
-      <c r="G28" s="0"/>
-      <c r="H28" s="0"/>
-      <c r="I28" s="0"/>
-      <c r="J28" s="0"/>
-      <c r="L28" s="0"/>
-      <c r="M28" s="0"/>
-      <c r="N28" s="0"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="0"/>
       <c r="O28" s="6"/>
       <c r="P28" s="6"/>
       <c r="Q28" s="6"/>
@@ -1480,27 +1425,25 @@
         <v>37</v>
       </c>
       <c r="B29" s="3" t="n">
+        <v>110.214918333333</v>
+      </c>
+      <c r="C29" s="3" t="n">
         <v>-7.76167166666667</v>
       </c>
-      <c r="C29" s="3" t="n">
-        <v>110.214918333333</v>
-      </c>
       <c r="D29" s="4" t="n">
+        <v>9141969.46732688</v>
+      </c>
+      <c r="E29" s="4" t="n">
         <v>413432.510138763</v>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>9141969.46732688</v>
       </c>
       <c r="F29" s="5" t="n">
         <v>98.5598718918457</v>
       </c>
-      <c r="G29" s="0"/>
-      <c r="H29" s="0"/>
-      <c r="I29" s="0"/>
-      <c r="J29" s="0"/>
-      <c r="L29" s="0"/>
-      <c r="M29" s="0"/>
-      <c r="N29" s="0"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="0"/>
       <c r="O29" s="6"/>
       <c r="P29" s="6"/>
       <c r="Q29" s="6"/>
@@ -1516,27 +1459,25 @@
         <v>38</v>
       </c>
       <c r="B30" s="3" t="n">
+        <v>110.213060467391</v>
+      </c>
+      <c r="C30" s="3" t="n">
         <v>-7.76939369418946</v>
       </c>
-      <c r="C30" s="3" t="n">
-        <v>110.213060467391</v>
-      </c>
       <c r="D30" s="4" t="n">
+        <v>9141115.33707188</v>
+      </c>
+      <c r="E30" s="4" t="n">
         <v>413229.223493991</v>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>9141115.33707188</v>
       </c>
       <c r="F30" s="5" t="n">
         <v>87.5125579833984</v>
       </c>
-      <c r="G30" s="0"/>
-      <c r="H30" s="0"/>
-      <c r="I30" s="0"/>
-      <c r="J30" s="0"/>
-      <c r="L30" s="0"/>
-      <c r="M30" s="0"/>
-      <c r="N30" s="0"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="0"/>
       <c r="O30" s="6"/>
       <c r="P30" s="6"/>
       <c r="Q30" s="6"/>
@@ -1552,27 +1493,25 @@
         <v>39</v>
       </c>
       <c r="B31" s="3" t="n">
+        <v>110.191381666667</v>
+      </c>
+      <c r="C31" s="3" t="n">
         <v>-7.76240666666667</v>
       </c>
-      <c r="C31" s="3" t="n">
-        <v>110.191381666667</v>
-      </c>
       <c r="D31" s="4" t="n">
+        <v>9141883.32974527</v>
+      </c>
+      <c r="E31" s="4" t="n">
         <v>410837.215986532</v>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>9141883.32974527</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>156.905288773438</v>
       </c>
-      <c r="G31" s="0"/>
-      <c r="H31" s="0"/>
-      <c r="I31" s="0"/>
-      <c r="J31" s="0"/>
-      <c r="L31" s="0"/>
-      <c r="M31" s="0"/>
-      <c r="N31" s="0"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="0"/>
       <c r="O31" s="6"/>
       <c r="P31" s="6"/>
       <c r="Q31" s="6"/>
@@ -1588,27 +1527,25 @@
         <v>40</v>
       </c>
       <c r="B32" s="3" t="n">
+        <v>110.2004</v>
+      </c>
+      <c r="C32" s="3" t="n">
         <v>-7.77120166666667</v>
       </c>
-      <c r="C32" s="3" t="n">
-        <v>110.2004</v>
-      </c>
       <c r="D32" s="4" t="n">
+        <v>9140912.8330531</v>
+      </c>
+      <c r="E32" s="4" t="n">
         <v>411833.524904229</v>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>9140912.8330531</v>
       </c>
       <c r="F32" s="5" t="n">
         <v>104.27709197998</v>
       </c>
-      <c r="G32" s="0"/>
-      <c r="H32" s="0"/>
-      <c r="I32" s="0"/>
-      <c r="J32" s="0"/>
-      <c r="L32" s="0"/>
-      <c r="M32" s="0"/>
-      <c r="N32" s="0"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="0"/>
       <c r="O32" s="6"/>
       <c r="P32" s="6"/>
       <c r="Q32" s="6"/>
@@ -1624,27 +1561,25 @@
         <v>41</v>
       </c>
       <c r="B33" s="3" t="n">
+        <v>110.190198333333</v>
+      </c>
+      <c r="C33" s="3" t="n">
         <v>-7.77023</v>
       </c>
-      <c r="C33" s="3" t="n">
-        <v>110.190198333333</v>
-      </c>
       <c r="D33" s="4" t="n">
+        <v>9141018.12503697</v>
+      </c>
+      <c r="E33" s="4" t="n">
         <v>410708.378725525</v>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>9141018.12503697</v>
       </c>
       <c r="F33" s="5" t="n">
         <v>180.585647583008</v>
       </c>
-      <c r="G33" s="0"/>
-      <c r="H33" s="0"/>
-      <c r="I33" s="0"/>
-      <c r="J33" s="0"/>
-      <c r="L33" s="0"/>
-      <c r="M33" s="0"/>
-      <c r="N33" s="0"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="0"/>
       <c r="O33" s="6"/>
       <c r="P33" s="6"/>
       <c r="Q33" s="6"/>
@@ -1660,27 +1595,25 @@
         <v>42</v>
       </c>
       <c r="B34" s="3" t="n">
+        <v>110.193580490479</v>
+      </c>
+      <c r="C34" s="3" t="n">
         <v>-7.74059808306336</v>
       </c>
-      <c r="C34" s="3" t="n">
-        <v>110.193580490479</v>
-      </c>
       <c r="D34" s="4" t="n">
+        <v>9144294.96716549</v>
+      </c>
+      <c r="E34" s="4" t="n">
         <v>411075.108599807</v>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>9144294.96716549</v>
       </c>
       <c r="F34" s="5" t="n">
         <v>184.640991210938</v>
       </c>
-      <c r="G34" s="0"/>
-      <c r="H34" s="0"/>
-      <c r="I34" s="0"/>
-      <c r="J34" s="0"/>
-      <c r="L34" s="0"/>
-      <c r="M34" s="0"/>
-      <c r="N34" s="0"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="0"/>
       <c r="O34" s="6"/>
       <c r="P34" s="6"/>
       <c r="Q34" s="6"/>
@@ -1696,27 +1629,25 @@
         <v>43</v>
       </c>
       <c r="B35" s="3" t="n">
+        <v>110.195285</v>
+      </c>
+      <c r="C35" s="3" t="n">
         <v>-7.729845</v>
       </c>
-      <c r="C35" s="3" t="n">
-        <v>110.195285</v>
-      </c>
       <c r="D35" s="4" t="n">
+        <v>9145484.19192017</v>
+      </c>
+      <c r="E35" s="4" t="n">
         <v>411260.831441595</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>9145484.19192017</v>
       </c>
       <c r="F35" s="5" t="n">
         <v>162.200424222168</v>
       </c>
-      <c r="G35" s="0"/>
-      <c r="H35" s="0"/>
-      <c r="I35" s="0"/>
-      <c r="J35" s="0"/>
-      <c r="L35" s="0"/>
-      <c r="M35" s="0"/>
-      <c r="N35" s="0"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="0"/>
       <c r="O35" s="6"/>
       <c r="P35" s="6"/>
       <c r="Q35" s="6"/>
@@ -1732,27 +1663,25 @@
         <v>44</v>
       </c>
       <c r="B36" s="3" t="n">
+        <v>110.203606666667</v>
+      </c>
+      <c r="C36" s="3" t="n">
         <v>-7.744135</v>
       </c>
-      <c r="C36" s="3" t="n">
-        <v>110.203606666667</v>
-      </c>
       <c r="D36" s="4" t="n">
+        <v>9143906.00678648</v>
+      </c>
+      <c r="E36" s="4" t="n">
         <v>412181.50944745</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>9143906.00678648</v>
       </c>
       <c r="F36" s="5" t="n">
         <v>103.0586736521</v>
       </c>
-      <c r="G36" s="0"/>
-      <c r="H36" s="0"/>
-      <c r="I36" s="0"/>
-      <c r="J36" s="0"/>
-      <c r="L36" s="0"/>
-      <c r="M36" s="0"/>
-      <c r="N36" s="0"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="0"/>
       <c r="O36" s="6"/>
       <c r="P36" s="6"/>
       <c r="Q36" s="6"/>
@@ -1768,27 +1697,25 @@
         <v>45</v>
       </c>
       <c r="B37" s="3" t="n">
+        <v>110.204931666667</v>
+      </c>
+      <c r="C37" s="3" t="n">
         <v>-7.747075</v>
       </c>
-      <c r="C37" s="3" t="n">
-        <v>110.204931666667</v>
-      </c>
       <c r="D37" s="4" t="n">
+        <v>9143581.23227445</v>
+      </c>
+      <c r="E37" s="4" t="n">
         <v>412328.234581498</v>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>9143581.23227445</v>
       </c>
       <c r="F37" s="5" t="n">
         <v>102.347770690918</v>
       </c>
-      <c r="G37" s="0"/>
-      <c r="H37" s="0"/>
-      <c r="I37" s="0"/>
-      <c r="J37" s="0"/>
-      <c r="L37" s="0"/>
-      <c r="M37" s="0"/>
-      <c r="N37" s="0"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="0"/>
       <c r="O37" s="6"/>
       <c r="P37" s="6"/>
       <c r="Q37" s="6"/>
@@ -1804,27 +1731,25 @@
         <v>46</v>
       </c>
       <c r="B38" s="3" t="n">
+        <v>110.205936666667</v>
+      </c>
+      <c r="C38" s="3" t="n">
         <v>-7.73901333333333</v>
       </c>
-      <c r="C38" s="3" t="n">
-        <v>110.205936666667</v>
-      </c>
       <c r="D38" s="4" t="n">
+        <v>9144472.74134048</v>
+      </c>
+      <c r="E38" s="4" t="n">
         <v>412437.397910906</v>
-      </c>
-      <c r="E38" s="4" t="n">
-        <v>9144472.74134048</v>
       </c>
       <c r="F38" s="5" t="n">
         <v>110.125648498535</v>
       </c>
-      <c r="G38" s="0"/>
-      <c r="H38" s="0"/>
-      <c r="I38" s="0"/>
-      <c r="J38" s="0"/>
-      <c r="L38" s="0"/>
-      <c r="M38" s="0"/>
-      <c r="N38" s="0"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="0"/>
       <c r="O38" s="6"/>
       <c r="P38" s="6"/>
       <c r="Q38" s="6"/>
@@ -1840,27 +1765,25 @@
         <v>47</v>
       </c>
       <c r="B39" s="3" t="n">
+        <v>110.23905</v>
+      </c>
+      <c r="C39" s="3" t="n">
         <v>-7.73855333333333</v>
       </c>
-      <c r="C39" s="3" t="n">
-        <v>110.23905</v>
-      </c>
       <c r="D39" s="4" t="n">
+        <v>9144530.2720892</v>
+      </c>
+      <c r="E39" s="4" t="n">
         <v>416088.978701437</v>
-      </c>
-      <c r="E39" s="4" t="n">
-        <v>9144530.2720892</v>
       </c>
       <c r="F39" s="5" t="n">
         <v>114.826515197754</v>
       </c>
-      <c r="G39" s="0"/>
-      <c r="H39" s="0"/>
-      <c r="I39" s="0"/>
-      <c r="J39" s="0"/>
-      <c r="L39" s="0"/>
-      <c r="M39" s="0"/>
-      <c r="N39" s="0"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="K39" s="0"/>
       <c r="O39" s="6"/>
       <c r="P39" s="6"/>
       <c r="Q39" s="6"/>
@@ -1876,27 +1799,25 @@
         <v>48</v>
       </c>
       <c r="B40" s="3" t="n">
+        <v>110.22523</v>
+      </c>
+      <c r="C40" s="3" t="n">
         <v>-7.736845</v>
       </c>
-      <c r="C40" s="3" t="n">
-        <v>110.22523</v>
-      </c>
       <c r="D40" s="4" t="n">
+        <v>9144716.39496686</v>
+      </c>
+      <c r="E40" s="4" t="n">
         <v>414564.594753531</v>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>9144716.39496686</v>
       </c>
       <c r="F40" s="5" t="n">
         <v>113.601337464844</v>
       </c>
-      <c r="G40" s="0"/>
-      <c r="H40" s="0"/>
-      <c r="I40" s="0"/>
-      <c r="J40" s="0"/>
-      <c r="L40" s="0"/>
-      <c r="M40" s="0"/>
-      <c r="N40" s="0"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="K40" s="0"/>
       <c r="O40" s="6"/>
       <c r="P40" s="6"/>
       <c r="Q40" s="6"/>
@@ -1912,27 +1833,25 @@
         <v>49</v>
       </c>
       <c r="B41" s="3" t="n">
+        <v>110.226703333333</v>
+      </c>
+      <c r="C41" s="3" t="n">
         <v>-7.730785</v>
       </c>
-      <c r="C41" s="3" t="n">
-        <v>110.226703333333</v>
-      </c>
       <c r="D41" s="4" t="n">
+        <v>9145386.68358463</v>
+      </c>
+      <c r="E41" s="4" t="n">
         <v>414725.854737934</v>
-      </c>
-      <c r="E41" s="4" t="n">
-        <v>9145386.68358463</v>
       </c>
       <c r="F41" s="5" t="n">
         <v>113.723861694336</v>
       </c>
-      <c r="G41" s="0"/>
-      <c r="H41" s="0"/>
-      <c r="I41" s="0"/>
-      <c r="J41" s="0"/>
-      <c r="L41" s="0"/>
-      <c r="M41" s="0"/>
-      <c r="N41" s="0"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="K41" s="0"/>
       <c r="O41" s="6"/>
       <c r="P41" s="6"/>
       <c r="Q41" s="6"/>
@@ -1948,27 +1867,25 @@
         <v>50</v>
       </c>
       <c r="B42" s="3" t="n">
+        <v>110.231738333333</v>
+      </c>
+      <c r="C42" s="3" t="n">
         <v>-7.73390833333333</v>
       </c>
-      <c r="C42" s="3" t="n">
-        <v>110.231738333333</v>
-      </c>
       <c r="D42" s="4" t="n">
+        <v>9145042.37340122</v>
+      </c>
+      <c r="E42" s="4" t="n">
         <v>415281.737319443</v>
-      </c>
-      <c r="E42" s="4" t="n">
-        <v>9145042.37340122</v>
       </c>
       <c r="F42" s="5" t="n">
         <v>118.082794189453</v>
       </c>
-      <c r="G42" s="0"/>
-      <c r="H42" s="0"/>
-      <c r="I42" s="0"/>
-      <c r="J42" s="0"/>
-      <c r="L42" s="0"/>
-      <c r="M42" s="0"/>
-      <c r="N42" s="0"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="K42" s="0"/>
       <c r="O42" s="6"/>
       <c r="P42" s="6"/>
       <c r="Q42" s="6"/>
@@ -1984,27 +1901,25 @@
         <v>51</v>
       </c>
       <c r="B43" s="3" t="n">
+        <v>110.23095</v>
+      </c>
+      <c r="C43" s="3" t="n">
         <v>-7.74343</v>
       </c>
-      <c r="C43" s="3" t="n">
-        <v>110.23095</v>
-      </c>
       <c r="D43" s="4" t="n">
+        <v>9143989.50253416</v>
+      </c>
+      <c r="E43" s="4" t="n">
         <v>415196.703429387</v>
-      </c>
-      <c r="E43" s="4" t="n">
-        <v>9143989.50253416</v>
       </c>
       <c r="F43" s="5" t="n">
         <v>117.907688356201</v>
       </c>
-      <c r="G43" s="0"/>
-      <c r="H43" s="0"/>
-      <c r="I43" s="0"/>
-      <c r="J43" s="0"/>
-      <c r="L43" s="0"/>
-      <c r="M43" s="0"/>
-      <c r="N43" s="0"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="0"/>
       <c r="O43" s="6"/>
       <c r="P43" s="6"/>
       <c r="Q43" s="6"/>
@@ -2020,27 +1935,25 @@
         <v>52</v>
       </c>
       <c r="B44" s="3" t="n">
+        <v>110.228493333333</v>
+      </c>
+      <c r="C44" s="3" t="n">
         <v>-7.74878666666667</v>
       </c>
-      <c r="C44" s="3" t="n">
-        <v>110.228493333333</v>
-      </c>
       <c r="D44" s="4" t="n">
+        <v>9143396.77905254</v>
+      </c>
+      <c r="E44" s="4" t="n">
         <v>414926.865360056</v>
-      </c>
-      <c r="E44" s="4" t="n">
-        <v>9143396.77905254</v>
       </c>
       <c r="F44" s="5" t="n">
         <v>96.8182830810547</v>
       </c>
-      <c r="G44" s="0"/>
-      <c r="H44" s="0"/>
-      <c r="I44" s="0"/>
-      <c r="J44" s="0"/>
-      <c r="L44" s="0"/>
-      <c r="M44" s="0"/>
-      <c r="N44" s="0"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="0"/>
       <c r="O44" s="6"/>
       <c r="P44" s="6"/>
       <c r="Q44" s="6"/>
@@ -2056,27 +1969,25 @@
         <v>53</v>
       </c>
       <c r="B45" s="3" t="n">
+        <v>110.227496730071</v>
+      </c>
+      <c r="C45" s="3" t="n">
         <v>-7.76058965774792</v>
       </c>
-      <c r="C45" s="3" t="n">
-        <v>110.227496730071</v>
-      </c>
       <c r="D45" s="4" t="n">
+        <v>9142091.64063808</v>
+      </c>
+      <c r="E45" s="4" t="n">
         <v>414819.338789763</v>
-      </c>
-      <c r="E45" s="4" t="n">
-        <v>9142091.64063808</v>
       </c>
       <c r="F45" s="5" t="n">
         <v>99.9816704658203</v>
       </c>
-      <c r="G45" s="0"/>
-      <c r="H45" s="0"/>
-      <c r="I45" s="0"/>
-      <c r="J45" s="0"/>
-      <c r="L45" s="0"/>
-      <c r="M45" s="0"/>
-      <c r="N45" s="0"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="0"/>
       <c r="O45" s="6"/>
       <c r="P45" s="6"/>
       <c r="Q45" s="6"/>
@@ -2092,27 +2003,25 @@
         <v>54</v>
       </c>
       <c r="B46" s="3" t="n">
+        <v>110.236688333333</v>
+      </c>
+      <c r="C46" s="3" t="n">
         <v>-7.75120845129024</v>
       </c>
-      <c r="C46" s="3" t="n">
-        <v>110.236688333333</v>
-      </c>
       <c r="D46" s="4" t="n">
+        <v>9143130.65923884</v>
+      </c>
+      <c r="E46" s="4" t="n">
         <v>415831.051589721</v>
-      </c>
-      <c r="E46" s="4" t="n">
-        <v>9143130.65923884</v>
       </c>
       <c r="F46" s="5" t="n">
         <v>116.905540466309</v>
       </c>
-      <c r="G46" s="0"/>
-      <c r="H46" s="0"/>
-      <c r="I46" s="0"/>
-      <c r="J46" s="0"/>
-      <c r="L46" s="0"/>
-      <c r="M46" s="0"/>
-      <c r="N46" s="0"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5"/>
+      <c r="K46" s="0"/>
       <c r="O46" s="6"/>
       <c r="P46" s="6"/>
       <c r="Q46" s="6"/>
@@ -2128,27 +2037,25 @@
         <v>55</v>
       </c>
       <c r="B47" s="3" t="n">
+        <v>110.242818333333</v>
+      </c>
+      <c r="C47" s="3" t="n">
         <v>-7.746465</v>
       </c>
-      <c r="C47" s="3" t="n">
-        <v>110.242818333333</v>
-      </c>
       <c r="D47" s="4" t="n">
+        <v>9143656.30307782</v>
+      </c>
+      <c r="E47" s="4" t="n">
         <v>416506.099035213</v>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>9143656.30307782</v>
       </c>
       <c r="F47" s="5" t="n">
         <v>110.521766662598</v>
       </c>
-      <c r="G47" s="0"/>
-      <c r="H47" s="0"/>
-      <c r="I47" s="0"/>
-      <c r="J47" s="0"/>
-      <c r="L47" s="0"/>
-      <c r="M47" s="0"/>
-      <c r="N47" s="0"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="K47" s="0"/>
       <c r="O47" s="6"/>
       <c r="P47" s="6"/>
       <c r="Q47" s="6"/>
@@ -2164,27 +2071,25 @@
         <v>56</v>
       </c>
       <c r="B48" s="3" t="n">
+        <v>110.247356666667</v>
+      </c>
+      <c r="C48" s="3" t="n">
         <v>-7.73529666666667</v>
       </c>
-      <c r="C48" s="3" t="n">
-        <v>110.247356666667</v>
-      </c>
       <c r="D48" s="4" t="n">
+        <v>9144891.95660562</v>
+      </c>
+      <c r="E48" s="4" t="n">
         <v>417004.381086391</v>
-      </c>
-      <c r="E48" s="4" t="n">
-        <v>9144891.95660562</v>
       </c>
       <c r="F48" s="5" t="n">
         <v>119.422584693359</v>
       </c>
-      <c r="G48" s="0"/>
-      <c r="H48" s="0"/>
-      <c r="I48" s="0"/>
-      <c r="J48" s="0"/>
-      <c r="L48" s="0"/>
-      <c r="M48" s="0"/>
-      <c r="N48" s="0"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="0"/>
       <c r="O48" s="6"/>
       <c r="P48" s="6"/>
       <c r="Q48" s="6"/>
@@ -2200,27 +2105,25 @@
         <v>57</v>
       </c>
       <c r="B49" s="3" t="n">
+        <v>110.258041666667</v>
+      </c>
+      <c r="C49" s="3" t="n">
         <v>-7.73211166666667</v>
       </c>
-      <c r="C49" s="3" t="n">
-        <v>110.258041666667</v>
-      </c>
       <c r="D49" s="4" t="n">
+        <v>9145246.15616601</v>
+      </c>
+      <c r="E49" s="4" t="n">
         <v>418182.090000391</v>
-      </c>
-      <c r="E49" s="4" t="n">
-        <v>9145246.15616601</v>
       </c>
       <c r="F49" s="5" t="n">
         <v>129.631423950195</v>
       </c>
-      <c r="G49" s="0"/>
-      <c r="H49" s="0"/>
-      <c r="I49" s="0"/>
-      <c r="J49" s="0"/>
-      <c r="L49" s="0"/>
-      <c r="M49" s="0"/>
-      <c r="N49" s="0"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="0"/>
       <c r="O49" s="6"/>
       <c r="P49" s="6"/>
       <c r="Q49" s="6"/>
@@ -2236,27 +2139,25 @@
         <v>58</v>
       </c>
       <c r="B50" s="3" t="n">
+        <v>110.257428333333</v>
+      </c>
+      <c r="C50" s="3" t="n">
         <v>-7.74282666666667</v>
       </c>
-      <c r="C50" s="3" t="n">
-        <v>110.257428333333</v>
-      </c>
       <c r="D50" s="4" t="n">
+        <v>9144061.39669829</v>
+      </c>
+      <c r="E50" s="4" t="n">
         <v>418116.519473534</v>
-      </c>
-      <c r="E50" s="4" t="n">
-        <v>9144061.39669829</v>
       </c>
       <c r="F50" s="5" t="n">
         <v>123.278053337646</v>
       </c>
-      <c r="G50" s="0"/>
-      <c r="H50" s="0"/>
-      <c r="I50" s="0"/>
-      <c r="J50" s="0"/>
-      <c r="L50" s="0"/>
-      <c r="M50" s="0"/>
-      <c r="N50" s="0"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="0"/>
       <c r="O50" s="6"/>
       <c r="P50" s="6"/>
       <c r="Q50" s="6"/>
@@ -2272,27 +2173,25 @@
         <v>59</v>
       </c>
       <c r="B51" s="3" t="n">
+        <v>110.251958148197</v>
+      </c>
+      <c r="C51" s="3" t="n">
         <v>-7.75552289561845</v>
       </c>
-      <c r="C51" s="3" t="n">
-        <v>110.251958148197</v>
-      </c>
       <c r="D51" s="4" t="n">
+        <v>9142656.65239711</v>
+      </c>
+      <c r="E51" s="4" t="n">
         <v>417515.759463108</v>
-      </c>
-      <c r="E51" s="4" t="n">
-        <v>9142656.65239711</v>
       </c>
       <c r="F51" s="5" t="n">
         <v>108.985710144043</v>
       </c>
-      <c r="G51" s="0"/>
-      <c r="H51" s="0"/>
-      <c r="I51" s="0"/>
-      <c r="J51" s="0"/>
-      <c r="L51" s="0"/>
-      <c r="M51" s="0"/>
-      <c r="N51" s="0"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="0"/>
       <c r="O51" s="6"/>
       <c r="P51" s="6"/>
       <c r="Q51" s="6"/>
@@ -2308,27 +2207,25 @@
         <v>60</v>
       </c>
       <c r="B52" s="3" t="n">
+        <v>110.24448</v>
+      </c>
+      <c r="C52" s="3" t="n">
         <v>-7.76307666666667</v>
       </c>
-      <c r="C52" s="3" t="n">
-        <v>110.24448</v>
-      </c>
       <c r="D52" s="4" t="n">
+        <v>9141820.05024063</v>
+      </c>
+      <c r="E52" s="4" t="n">
         <v>416692.6081601</v>
-      </c>
-      <c r="E52" s="4" t="n">
-        <v>9141820.05024063</v>
       </c>
       <c r="F52" s="5" t="n">
         <v>109.82119761499</v>
       </c>
-      <c r="G52" s="0"/>
-      <c r="H52" s="0"/>
-      <c r="I52" s="0"/>
-      <c r="J52" s="0"/>
-      <c r="L52" s="0"/>
-      <c r="M52" s="0"/>
-      <c r="N52" s="0"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="0"/>
       <c r="O52" s="6"/>
       <c r="P52" s="6"/>
       <c r="Q52" s="6"/>
@@ -2344,27 +2241,25 @@
         <v>61</v>
       </c>
       <c r="B53" s="3" t="n">
+        <v>110.208526</v>
+      </c>
+      <c r="C53" s="3" t="n">
         <v>-7.720965</v>
       </c>
-      <c r="C53" s="3" t="n">
-        <v>110.208526</v>
-      </c>
       <c r="D53" s="4" t="n">
+        <v>9146468.70371187</v>
+      </c>
+      <c r="E53" s="4" t="n">
         <v>412719.237582945</v>
-      </c>
-      <c r="E53" s="4" t="n">
-        <v>9146468.70371187</v>
       </c>
       <c r="F53" s="5" t="n">
         <v>167.074172973633</v>
       </c>
-      <c r="G53" s="0"/>
-      <c r="H53" s="0"/>
-      <c r="I53" s="0"/>
-      <c r="J53" s="0"/>
-      <c r="L53" s="0"/>
-      <c r="M53" s="0"/>
-      <c r="N53" s="0"/>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="K53" s="0"/>
       <c r="O53" s="6"/>
       <c r="P53" s="6"/>
       <c r="Q53" s="6"/>
@@ -2380,27 +2275,25 @@
         <v>62</v>
       </c>
       <c r="B54" s="3" t="n">
+        <v>110.203814961153</v>
+      </c>
+      <c r="C54" s="3" t="n">
         <v>-7.72067601534982</v>
       </c>
-      <c r="C54" s="3" t="n">
-        <v>110.203814961153</v>
-      </c>
       <c r="D54" s="4" t="n">
+        <v>9146499.68683582</v>
+      </c>
+      <c r="E54" s="4" t="n">
         <v>412199.630010951</v>
-      </c>
-      <c r="E54" s="4" t="n">
-        <v>9146499.68683582</v>
       </c>
       <c r="F54" s="5" t="n">
         <v>216.702954231122</v>
       </c>
-      <c r="G54" s="0"/>
-      <c r="H54" s="0"/>
-      <c r="I54" s="0"/>
-      <c r="J54" s="0"/>
-      <c r="L54" s="0"/>
-      <c r="M54" s="0"/>
-      <c r="N54" s="0"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="K54" s="0"/>
       <c r="O54" s="6"/>
       <c r="P54" s="6"/>
       <c r="Q54" s="6"/>
@@ -2416,27 +2309,25 @@
         <v>63</v>
       </c>
       <c r="B55" s="3" t="n">
+        <v>110.197189867159</v>
+      </c>
+      <c r="C55" s="3" t="n">
         <v>-7.71763077414723</v>
       </c>
-      <c r="C55" s="3" t="n">
-        <v>110.197189867159</v>
-      </c>
       <c r="D55" s="4" t="n">
+        <v>9146835.00078957</v>
+      </c>
+      <c r="E55" s="4" t="n">
         <v>411468.359016951</v>
-      </c>
-      <c r="E55" s="4" t="n">
-        <v>9146835.00078957</v>
       </c>
       <c r="F55" s="5" t="n">
         <v>357.373662546629</v>
       </c>
-      <c r="G55" s="0"/>
-      <c r="H55" s="0"/>
-      <c r="I55" s="0"/>
-      <c r="J55" s="0"/>
-      <c r="L55" s="0"/>
-      <c r="M55" s="0"/>
-      <c r="N55" s="0"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="K55" s="0"/>
       <c r="O55" s="6"/>
       <c r="P55" s="6"/>
       <c r="Q55" s="6"/>
@@ -2452,27 +2343,25 @@
         <v>64</v>
       </c>
       <c r="B56" s="3" t="n">
+        <v>110.211681409509</v>
+      </c>
+      <c r="C56" s="3" t="n">
         <v>-7.7161896198009</v>
       </c>
-      <c r="C56" s="3" t="n">
-        <v>110.211681409509</v>
-      </c>
       <c r="D56" s="4" t="n">
+        <v>9146997.31539322</v>
+      </c>
+      <c r="E56" s="4" t="n">
         <v>413066.249877809</v>
-      </c>
-      <c r="E56" s="4" t="n">
-        <v>9146997.31539322</v>
       </c>
       <c r="F56" s="5" t="n">
         <v>132.581039268066</v>
       </c>
-      <c r="G56" s="0"/>
-      <c r="H56" s="0"/>
-      <c r="I56" s="0"/>
-      <c r="J56" s="0"/>
-      <c r="L56" s="0"/>
-      <c r="M56" s="0"/>
-      <c r="N56" s="0"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5"/>
+      <c r="K56" s="0"/>
       <c r="O56" s="6"/>
       <c r="P56" s="6"/>
       <c r="Q56" s="6"/>
@@ -2488,27 +2377,25 @@
         <v>65</v>
       </c>
       <c r="B57" s="3" t="n">
+        <v>110.2052347</v>
+      </c>
+      <c r="C57" s="3" t="n">
         <v>-7.7136595</v>
       </c>
-      <c r="C57" s="3" t="n">
-        <v>110.2052347</v>
-      </c>
       <c r="D57" s="4" t="n">
+        <v>9147275.72752503</v>
+      </c>
+      <c r="E57" s="4" t="n">
         <v>412354.758300737</v>
-      </c>
-      <c r="E57" s="4" t="n">
-        <v>9147275.72752503</v>
       </c>
       <c r="F57" s="5" t="n">
         <v>263.128784376953</v>
       </c>
-      <c r="G57" s="0"/>
-      <c r="H57" s="0"/>
-      <c r="I57" s="0"/>
-      <c r="J57" s="0"/>
-      <c r="L57" s="0"/>
-      <c r="M57" s="0"/>
-      <c r="N57" s="0"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="5"/>
+      <c r="K57" s="0"/>
       <c r="O57" s="6"/>
       <c r="P57" s="6"/>
       <c r="Q57" s="6"/>
@@ -2524,27 +2411,25 @@
         <v>66</v>
       </c>
       <c r="B58" s="3" t="n">
+        <v>110.195875</v>
+      </c>
+      <c r="C58" s="3" t="n">
         <v>-7.710344</v>
       </c>
-      <c r="C58" s="3" t="n">
-        <v>110.195875</v>
-      </c>
       <c r="D58" s="4" t="n">
+        <v>9147640.35790618</v>
+      </c>
+      <c r="E58" s="4" t="n">
         <v>411321.832155814</v>
-      </c>
-      <c r="E58" s="4" t="n">
-        <v>9147640.35790618</v>
       </c>
       <c r="F58" s="5" t="n">
         <v>386.825546503906</v>
       </c>
-      <c r="G58" s="0"/>
-      <c r="H58" s="0"/>
-      <c r="I58" s="0"/>
-      <c r="J58" s="0"/>
-      <c r="L58" s="0"/>
-      <c r="M58" s="0"/>
-      <c r="N58" s="0"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="5"/>
+      <c r="K58" s="0"/>
       <c r="O58" s="6"/>
       <c r="P58" s="6"/>
       <c r="Q58" s="6"/>
@@ -2560,27 +2445,25 @@
         <v>67</v>
       </c>
       <c r="B59" s="3" t="n">
+        <v>110.1875488</v>
+      </c>
+      <c r="C59" s="3" t="n">
         <v>-7.71324527</v>
       </c>
-      <c r="C59" s="3" t="n">
-        <v>110.1875488</v>
-      </c>
       <c r="D59" s="4" t="n">
+        <v>9147317.85298952</v>
+      </c>
+      <c r="E59" s="4" t="n">
         <v>410404.177428969</v>
-      </c>
-      <c r="E59" s="4" t="n">
-        <v>9147317.85298952</v>
       </c>
       <c r="F59" s="5" t="n">
         <v>390.998794449219</v>
       </c>
-      <c r="G59" s="0"/>
-      <c r="H59" s="0"/>
-      <c r="I59" s="0"/>
-      <c r="J59" s="0"/>
-      <c r="L59" s="0"/>
-      <c r="M59" s="0"/>
-      <c r="N59" s="0"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="5"/>
+      <c r="K59" s="0"/>
       <c r="O59" s="6"/>
       <c r="P59" s="6"/>
       <c r="Q59" s="6"/>
@@ -2596,27 +2479,25 @@
         <v>68</v>
       </c>
       <c r="B60" s="3" t="n">
+        <v>110.1857459</v>
+      </c>
+      <c r="C60" s="3" t="n">
         <v>-7.7193371</v>
       </c>
-      <c r="C60" s="3" t="n">
-        <v>110.1857459</v>
-      </c>
       <c r="D60" s="4" t="n">
+        <v>9146643.95597048</v>
+      </c>
+      <c r="E60" s="4" t="n">
         <v>410206.628769814</v>
-      </c>
-      <c r="E60" s="4" t="n">
-        <v>9146643.95597048</v>
       </c>
       <c r="F60" s="5" t="n">
         <v>431.893676511719</v>
       </c>
-      <c r="G60" s="0"/>
-      <c r="H60" s="0"/>
-      <c r="I60" s="0"/>
-      <c r="J60" s="0"/>
-      <c r="L60" s="0"/>
-      <c r="M60" s="0"/>
-      <c r="N60" s="0"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+      <c r="I60" s="5"/>
+      <c r="J60" s="5"/>
+      <c r="K60" s="0"/>
       <c r="O60" s="6"/>
       <c r="P60" s="6"/>
       <c r="Q60" s="6"/>
@@ -2632,27 +2513,25 @@
         <v>69</v>
       </c>
       <c r="B61" s="3" t="n">
+        <v>110.1882405</v>
+      </c>
+      <c r="C61" s="3" t="n">
         <v>-7.724188431</v>
       </c>
-      <c r="C61" s="3" t="n">
-        <v>110.1882405</v>
-      </c>
       <c r="D61" s="4" t="n">
+        <v>9146108.1130678</v>
+      </c>
+      <c r="E61" s="4" t="n">
         <v>410482.764387807</v>
-      </c>
-      <c r="E61" s="4" t="n">
-        <v>9146108.1130678</v>
       </c>
       <c r="F61" s="5" t="n">
         <v>314.894424208008</v>
       </c>
-      <c r="G61" s="0"/>
-      <c r="H61" s="0"/>
-      <c r="I61" s="0"/>
-      <c r="J61" s="0"/>
-      <c r="L61" s="0"/>
-      <c r="M61" s="0"/>
-      <c r="N61" s="0"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="5"/>
+      <c r="K61" s="0"/>
       <c r="O61" s="6"/>
       <c r="P61" s="6"/>
       <c r="Q61" s="6"/>

</xml_diff>